<commit_message>
Fix: Resolucion de conflicto en Transformer V1
</commit_message>
<xml_diff>
--- a/01_EXTRACCION DE DATOS/solicitud.xlsx
+++ b/01_EXTRACCION DE DATOS/solicitud.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jairi\OneDrive\Escritorio\TFM\CODIGOS EXTRACCION\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jairi\OneDrive\Escritorio\TFM\01_EXTRACCION DE DATOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1E38013-20E4-4631-AC31-6B2128E50D84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08C43877-9E27-4DC3-A1F7-60764440B60C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{559FDFCD-B43D-46E1-B413-71FA7BBCB967}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{559FDFCD-B43D-46E1-B413-71FA7BBCB967}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="6">
   <si>
     <t>Reference</t>
   </si>
@@ -50,63 +50,10 @@
     <t>mov_type</t>
   </si>
   <si>
-    <t>TABUENCA01-45</t>
-  </si>
-  <si>
-    <t>Walking_Ref</t>
-  </si>
-  <si>
-    <t>01912299X-118</t>
-  </si>
-  <si>
-    <t>Walking_Larga</t>
-  </si>
-  <si>
-    <t>02548893X-118</t>
-  </si>
-  <si>
-    <t>Walking_Noche</t>
-  </si>
-  <si>
-    <t>9 min de marcha continua</t>
-  </si>
-  <si>
-    <t>JOM20240407-104</t>
-  </si>
-  <si>
-    <t>Walking_JOM</t>
-  </si>
-  <si>
-    <t>Paciente distinto (2 min)</t>
-  </si>
-  <si>
-    <t>MGM-202406-79</t>
-  </si>
-  <si>
-    <t>Walking_MGM</t>
-  </si>
-  <si>
-    <t>5 min de marcha</t>
-  </si>
-  <si>
-    <r>
-      <t>15 min de caminata</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (ver fatiga)</t>
-    </r>
-  </si>
-  <si>
     <t>tag</t>
   </si>
   <si>
-    <t>base (2 min)</t>
+    <t>JASAHUG010-85</t>
   </si>
 </sst>
 </file>
@@ -143,7 +90,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -166,22 +113,42 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="22" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="22" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -516,7 +483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17D7DD9F-7BAB-48FB-BBA2-7BC418A185A9}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="14.83203125" style="1" customWidth="1"/>
@@ -526,106 +493,141 @@
     <col min="5" max="5" width="16.58203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.5" thickBot="1">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:7" ht="14.5" thickBot="1">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>18</v>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="28.5" thickBot="1">
+    <row r="2" spans="1:7" ht="28">
       <c r="A2" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="4">
-        <v>45407.677430555559</v>
+        <v>46015.410601851851</v>
       </c>
       <c r="C2" s="4">
-        <v>45407.678819444445</v>
-      </c>
-      <c r="D2" s="2" t="s">
+        <v>46015.443148148152</v>
+      </c>
+      <c r="D2" s="5">
+        <v>1</v>
+      </c>
+      <c r="E2" s="5"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6">
+        <f>+(C2-B2)*24*60</f>
+        <v>46.866666673449799</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="28">
+      <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>19</v>
+      <c r="B3" s="7">
+        <v>46015.443159722221</v>
+      </c>
+      <c r="C3" s="7">
+        <v>46015.45380787037</v>
+      </c>
+      <c r="D3" s="6">
+        <v>0</v>
+      </c>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6">
+        <f>+(C3-B3)*24*60</f>
+        <v>15.333333334419876</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="42.5" thickBot="1">
-      <c r="A3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="4">
-        <v>45716.778113425928</v>
-      </c>
-      <c r="C3" s="4">
-        <v>45716.789027777777</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>17</v>
+    <row r="4" spans="1:7" ht="28">
+      <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="7">
+        <v>46015.453819444447</v>
+      </c>
+      <c r="C4" s="7">
+        <v>46015.456770833334</v>
+      </c>
+      <c r="D4" s="6">
+        <v>1</v>
+      </c>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6">
+        <f>+(C4-B4)*24*60</f>
+        <v>4.2499999981373549</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="42.5" thickBot="1">
-      <c r="A4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="4">
-        <v>45716.956412037034</v>
-      </c>
-      <c r="C4" s="4">
-        <v>45716.963009259256</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>10</v>
+    <row r="5" spans="1:7" ht="28">
+      <c r="A5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="7">
+        <v>46015.456770833334</v>
+      </c>
+      <c r="C5" s="7">
+        <v>46015.457152777781</v>
+      </c>
+      <c r="D5" s="6">
+        <v>0</v>
+      </c>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6">
+        <f>+(C5-B5)*24*60</f>
+        <v>0.55000000284053385</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="42.5" thickBot="1">
-      <c r="A5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="4">
-        <v>45389.432650462964</v>
-      </c>
-      <c r="C5" s="4">
-        <v>45389.434039351851</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>13</v>
+    <row r="6" spans="1:7" ht="28">
+      <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7">
+        <v>46015.457152777781</v>
+      </c>
+      <c r="C6" s="7">
+        <v>46015.463402777779</v>
+      </c>
+      <c r="D6" s="6">
+        <v>1</v>
+      </c>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6">
+        <f>+(C6-B6)*24*60</f>
+        <v>8.9999999979045242</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="28.5" thickBot="1">
-      <c r="A6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="4">
-        <v>45459.55976851852</v>
-      </c>
-      <c r="C6" s="4">
-        <v>45459.563240740739</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>16</v>
+    <row r="7" spans="1:7" ht="28">
+      <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4">
+        <v>46015.404756944445</v>
+      </c>
+      <c r="C7" s="4">
+        <v>46015.410590277781</v>
+      </c>
+      <c r="D7" s="6">
+        <v>0</v>
+      </c>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6">
+        <f>+(C7-B7)*24*60</f>
+        <v>8.40000000433065</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización de scripts de extracción, limpieza y entrenamiento; inclusión de módulo de inferencia sliding
</commit_message>
<xml_diff>
--- a/01_EXTRACCION DE DATOS/solicitud.xlsx
+++ b/01_EXTRACCION DE DATOS/solicitud.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jairi\OneDrive\Escritorio\TFM\01_EXTRACCION DE DATOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08C43877-9E27-4DC3-A1F7-60764440B60C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3C01B69-7386-4427-A747-B03C7E0E4C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{559FDFCD-B43D-46E1-B413-71FA7BBCB967}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="96">
   <si>
     <t>Reference</t>
   </si>
@@ -54,13 +55,283 @@
   </si>
   <si>
     <t>JASAHUG010-85</t>
+  </si>
+  <si>
+    <t>TABUENCA01-45</t>
+  </si>
+  <si>
+    <t>25/04/2024 16:15</t>
+  </si>
+  <si>
+    <t>25/04/2024 16:17</t>
+  </si>
+  <si>
+    <t>2 min</t>
+  </si>
+  <si>
+    <t>25/04/2024 16:48</t>
+  </si>
+  <si>
+    <t>20 seg reposo</t>
+  </si>
+  <si>
+    <t>01912299X-118</t>
+  </si>
+  <si>
+    <t>24/04/2024 11:23</t>
+  </si>
+  <si>
+    <t>24/04/2024 11:59</t>
+  </si>
+  <si>
+    <t>36 min reposo</t>
+  </si>
+  <si>
+    <t>24/04/2024 12:00</t>
+  </si>
+  <si>
+    <t>1min caminata</t>
+  </si>
+  <si>
+    <t>24/04/2024 12:18</t>
+  </si>
+  <si>
+    <t>24/04/2024 12:28</t>
+  </si>
+  <si>
+    <t>No marcha</t>
+  </si>
+  <si>
+    <t>28/02/2025 18:40</t>
+  </si>
+  <si>
+    <t>28/02/2025 18:56</t>
+  </si>
+  <si>
+    <t>15 min de caminata</t>
+  </si>
+  <si>
+    <t>24/04/2024 11:21</t>
+  </si>
+  <si>
+    <t>24/04/2024 11:22</t>
+  </si>
+  <si>
+    <t>1 min Caminata</t>
+  </si>
+  <si>
+    <t>24/04/2024 10:51</t>
+  </si>
+  <si>
+    <t>24/04/2024 11:01</t>
+  </si>
+  <si>
+    <t>02548893X-118</t>
+  </si>
+  <si>
+    <t>28/02/2025 22:57</t>
+  </si>
+  <si>
+    <t>28/02/2025 23:06</t>
+  </si>
+  <si>
+    <t>9 min de marcha continua</t>
+  </si>
+  <si>
+    <t>04845288Q-121</t>
+  </si>
+  <si>
+    <t>caminata</t>
+  </si>
+  <si>
+    <t>no marcha se mueve</t>
+  </si>
+  <si>
+    <t>marcha</t>
+  </si>
+  <si>
+    <t>JOM20240407-104</t>
+  </si>
+  <si>
+    <t>Paciente distinto (2 min)</t>
+  </si>
+  <si>
+    <t>MGM-202406-79</t>
+  </si>
+  <si>
+    <t>16/06/2024 13:26</t>
+  </si>
+  <si>
+    <t>16/06/2024 13:31</t>
+  </si>
+  <si>
+    <t>5 min de marcha</t>
+  </si>
+  <si>
+    <t>05323975G-108</t>
+  </si>
+  <si>
+    <t>no marcha</t>
+  </si>
+  <si>
+    <t>05447093A-110</t>
+  </si>
+  <si>
+    <t>marcha con unos breves periodos raros</t>
+  </si>
+  <si>
+    <t>marcha clara</t>
+  </si>
+  <si>
+    <t>2025-CJ1-SJ2-49</t>
+  </si>
+  <si>
+    <t>15/05/2025 19:58</t>
+  </si>
+  <si>
+    <t>15/05/2025 20:05</t>
+  </si>
+  <si>
+    <t>15/05/2025 20:07</t>
+  </si>
+  <si>
+    <t>15/05/2025 20:17</t>
+  </si>
+  <si>
+    <t>15/05/2025 20:25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no marcha </t>
+  </si>
+  <si>
+    <t>2025-CJ2-SJ2-50</t>
+  </si>
+  <si>
+    <t>15/05/2025 20:44</t>
+  </si>
+  <si>
+    <t>15/05/2025 20:50</t>
+  </si>
+  <si>
+    <t>15/05/2025 21:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marcha </t>
+  </si>
+  <si>
+    <t>20266247G-97</t>
+  </si>
+  <si>
+    <t>28/03/2025 18:56</t>
+  </si>
+  <si>
+    <t>28/03/2025 18:59</t>
+  </si>
+  <si>
+    <t>28/03/2025 19:09</t>
+  </si>
+  <si>
+    <t>Marcha perfecta</t>
+  </si>
+  <si>
+    <t>28/03/2025 19:14</t>
+  </si>
+  <si>
+    <t>28/03/2025 19:16</t>
+  </si>
+  <si>
+    <t>28/03/2025 19:26</t>
+  </si>
+  <si>
+    <t>53471345W-118</t>
+  </si>
+  <si>
+    <t>16/04/2024 7:50</t>
+  </si>
+  <si>
+    <t>16/04/2024 8:14</t>
+  </si>
+  <si>
+    <t>16/04/2024 8:16</t>
+  </si>
+  <si>
+    <t>16/04/2024 8:30</t>
+  </si>
+  <si>
+    <t>16/04/2024 8:32</t>
+  </si>
+  <si>
+    <t>16/04/2024 9:02</t>
+  </si>
+  <si>
+    <t>16/04/2024 9:52</t>
+  </si>
+  <si>
+    <t>77370299R-115</t>
+  </si>
+  <si>
+    <t>EPGHUG006-25</t>
+  </si>
+  <si>
+    <t>13/12/2025 10:33</t>
+  </si>
+  <si>
+    <t>13/12/2025 10:40</t>
+  </si>
+  <si>
+    <t>buena marcha</t>
+  </si>
+  <si>
+    <t>13/12/2025 10:44</t>
+  </si>
+  <si>
+    <t>13/12/2025 10:55</t>
+  </si>
+  <si>
+    <t>13/12/2025 11:22</t>
+  </si>
+  <si>
+    <t>13/12/2025 11:48</t>
+  </si>
+  <si>
+    <t>JCGMHUG007-73</t>
+  </si>
+  <si>
+    <t>17/12/2025 5:26</t>
+  </si>
+  <si>
+    <t>17/12/2025 5:27</t>
+  </si>
+  <si>
+    <t>17/12/2025 5:29</t>
+  </si>
+  <si>
+    <t>17/12/2025 5:32</t>
+  </si>
+  <si>
+    <t>17/12/2025 6:54</t>
+  </si>
+  <si>
+    <t>17/12/2025 6:56</t>
+  </si>
+  <si>
+    <t>17/12/2025 7:11</t>
+  </si>
+  <si>
+    <t>17/12/2025 7:24</t>
+  </si>
+  <si>
+    <t>RSBHUGOO5-11</t>
+  </si>
+  <si>
+    <t>duracion</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -81,6 +352,33 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -90,7 +388,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -128,11 +426,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -149,6 +456,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -483,7 +799,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17D7DD9F-7BAB-48FB-BBA2-7BC418A185A9}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="14.83203125" style="1" customWidth="1"/>
@@ -509,8 +825,1015 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="G1" s="14" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="2" spans="1:7" ht="28">
+      <c r="A2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="5">
+        <v>1</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8">
+        <v>1.9999999959999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="28">
+      <c r="A3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="5">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8">
+        <v>0.34999999799999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="5">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8">
+        <v>36.450000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="5">
+        <v>1</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8">
+        <v>0.783333328</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="5">
+        <v>0</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8">
+        <v>9.6999999940000006</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="28">
+      <c r="A7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="5">
+        <v>1</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8">
+        <v>15.71666666</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="5">
+        <v>1</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8">
+        <v>0.88333333000000003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="5">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8">
+        <v>9.8333333270000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="28">
+      <c r="A10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="5">
+        <v>1</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="4">
+        <v>45660.488888888889</v>
+      </c>
+      <c r="C11" s="4">
+        <v>45660.488888888889</v>
+      </c>
+      <c r="D11" s="5">
+        <v>1</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8">
+        <v>0.73333000000000004</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="28">
+      <c r="A12" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="4">
+        <v>45660.489583333336</v>
+      </c>
+      <c r="C12" s="4">
+        <v>45660.493055555555</v>
+      </c>
+      <c r="D12" s="5">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8">
+        <v>5.6833299999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="4">
+        <v>45660.493055555555</v>
+      </c>
+      <c r="C13" s="4">
+        <v>45660.494444444441</v>
+      </c>
+      <c r="D13" s="5">
+        <v>1</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8">
+        <v>1.1499999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="28">
+      <c r="A14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="4">
+        <v>45477.432638888888</v>
+      </c>
+      <c r="C14" s="4">
+        <v>45477.434027777781</v>
+      </c>
+      <c r="D14" s="5">
+        <v>1</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" s="5">
+        <v>1</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="10">
+        <v>45965.709722222222</v>
+      </c>
+      <c r="C16" s="10">
+        <v>45965.709722222222</v>
+      </c>
+      <c r="D16" s="5">
+        <v>1</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8">
+        <v>0.61667000000000005</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="10">
+        <v>45965.710416666669</v>
+      </c>
+      <c r="C17" s="10">
+        <v>45965.710416666669</v>
+      </c>
+      <c r="D17" s="5">
+        <v>1</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" s="10">
+        <v>45965.716666666667</v>
+      </c>
+      <c r="C18" s="10">
+        <v>45965.717361111114</v>
+      </c>
+      <c r="D18" s="5">
+        <v>0</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8">
+        <v>0.31667000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="10">
+        <v>45965.719444444447</v>
+      </c>
+      <c r="C19" s="10">
+        <v>45965.719444444447</v>
+      </c>
+      <c r="D19" s="5">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="42">
+      <c r="A20" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="10">
+        <v>45540.472916666666</v>
+      </c>
+      <c r="C20" s="10">
+        <v>45540.476388888892</v>
+      </c>
+      <c r="D20" s="5">
+        <v>1</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8">
+        <v>4.9833299999999996</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B21" s="10">
+        <v>45540.435416666667</v>
+      </c>
+      <c r="C21" s="10">
+        <v>45540.47152777778</v>
+      </c>
+      <c r="D21" s="12">
+        <v>0</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8">
+        <v>52.333329999999997</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="10">
+        <v>45540.523611111108</v>
+      </c>
+      <c r="C22" s="10">
+        <v>45540.524305555555</v>
+      </c>
+      <c r="D22" s="12">
+        <v>1</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8">
+        <v>0.83333000000000002</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" s="10">
+        <v>45540.524305555555</v>
+      </c>
+      <c r="C23" s="10">
+        <v>45540.53125</v>
+      </c>
+      <c r="D23" s="12">
+        <v>0</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8">
+        <v>10.716670000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" s="12">
+        <v>0</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8">
+        <v>7.3833299999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25" s="12">
+        <v>1</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8">
+        <v>1.6333299999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D26" s="12">
+        <v>0</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8">
+        <v>8.0833300000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D27" s="12">
+        <v>0</v>
+      </c>
+      <c r="E27" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8">
+        <v>5.9833299999999996</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D28" s="12">
+        <v>1</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8">
+        <v>0.33333000000000002</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="D29" s="12">
+        <v>0</v>
+      </c>
+      <c r="E29" s="12"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D30" s="12">
+        <v>1</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8">
+        <v>9.9499999999999993</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D31" s="12">
+        <v>1</v>
+      </c>
+      <c r="E31" s="12"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8">
+        <v>-498895.31666999997</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D32" s="12">
+        <v>0</v>
+      </c>
+      <c r="E32" s="12"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D33" s="12">
+        <v>1</v>
+      </c>
+      <c r="E33" s="12"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8">
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="D34" s="12">
+        <v>0</v>
+      </c>
+      <c r="E34" s="12"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="D35" s="12">
+        <v>1</v>
+      </c>
+      <c r="E35" s="12"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8">
+        <v>2.76667</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="D36" s="12">
+        <v>1</v>
+      </c>
+      <c r="E36" s="12"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D37" s="12">
+        <v>0</v>
+      </c>
+      <c r="E37" s="12"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8">
+        <v>49.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B38" s="10">
+        <v>45393.344444444447</v>
+      </c>
+      <c r="C38" s="10">
+        <v>45393.356249999997</v>
+      </c>
+      <c r="D38" s="12">
+        <v>0</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="D39" s="12">
+        <v>1</v>
+      </c>
+      <c r="E39" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8">
+        <v>6.05</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B40" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C40" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="D40" s="12">
+        <v>0</v>
+      </c>
+      <c r="E40" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="F40" s="8"/>
+      <c r="G40" s="8">
+        <v>10.283329999999999</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B41" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="D41" s="12">
+        <v>0</v>
+      </c>
+      <c r="E41" s="12"/>
+      <c r="F41" s="8"/>
+      <c r="G41" s="8">
+        <v>25.45</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B42" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="D42" s="12">
+        <v>1</v>
+      </c>
+      <c r="E42" s="12"/>
+      <c r="F42" s="8"/>
+      <c r="G42" s="8">
+        <v>1.55</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B43" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D43" s="12">
+        <v>0</v>
+      </c>
+      <c r="E43" s="12"/>
+      <c r="F43" s="8"/>
+      <c r="G43" s="8">
+        <v>2.48333</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B44" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="C44" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="D44" s="12">
+        <v>1</v>
+      </c>
+      <c r="E44" s="12"/>
+      <c r="F44" s="8"/>
+      <c r="G44" s="8">
+        <v>1.2166699999999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B45" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D45" s="12">
+        <v>0</v>
+      </c>
+      <c r="E45" s="12"/>
+      <c r="F45" s="8"/>
+      <c r="G45" s="8">
+        <v>13.35</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="B46" s="10">
+        <v>45820.550694444442</v>
+      </c>
+      <c r="C46" s="10">
+        <v>45820.551388888889</v>
+      </c>
+      <c r="D46" s="12">
+        <v>1</v>
+      </c>
+      <c r="E46" s="12"/>
+      <c r="F46" s="8"/>
+      <c r="G46" s="8">
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="A47" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="B47" s="10">
+        <v>45820.557638888888</v>
+      </c>
+      <c r="C47" s="10">
+        <v>45820.558333333334</v>
+      </c>
+      <c r="D47" s="12">
+        <v>1</v>
+      </c>
+      <c r="E47" s="12"/>
+      <c r="F47" s="8"/>
+      <c r="G47" s="8">
+        <v>1.0833299999999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="B48" s="10">
+        <v>45820.570138888892</v>
+      </c>
+      <c r="C48" s="10">
+        <v>45820.572222222225</v>
+      </c>
+      <c r="D48" s="12">
+        <v>0</v>
+      </c>
+      <c r="E48" s="12"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="8">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="B49" s="10">
+        <v>45820.574305555558</v>
+      </c>
+      <c r="C49" s="10">
+        <v>45820.584027777775</v>
+      </c>
+      <c r="D49" s="12">
+        <v>0</v>
+      </c>
+      <c r="E49" s="12"/>
+      <c r="F49" s="8"/>
+      <c r="G49" s="8">
+        <v>14.41667</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3C2A3F5-64C2-485E-A87E-AD3BE87A0A2E}">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
+  <cols>
+    <col min="1" max="7" width="17.08203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="14.5" thickBot="1">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>

</xml_diff>